<commit_message>
fix: improve CAD audit scanning and normalized matching
</commit_message>
<xml_diff>
--- a/documents_bin/词库收集.xlsx
+++ b/documents_bin/词库收集.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\project\auto-fanban-pre\documents_bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0432AC2-A136-4C28-9BF5-C4775F538A9E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278E9DDB-B57D-4462-AAA7-66A8861FF486}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="4350" windowWidth="28800" windowHeight="15315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="289">
   <si>
     <t>项目号</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -934,6 +934,15 @@
   </si>
   <si>
     <t>CP05JT0407</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">浙江金七门核电厂 1、2 号 机 组
+</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>江苏徐圩核能供热发电厂一期工程</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1092,7 +1101,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1135,6 +1144,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1143,6 +1155,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1426,13 +1441,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O116"/>
+  <dimension ref="A1:O117"/>
   <sheetFormatPr defaultRowHeight="20.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
     <col min="2" max="6" width="20.625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="26" style="2" customWidth="1"/>
-    <col min="8" max="8" width="23.75" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="42.125" style="2" customWidth="1"/>
     <col min="9" max="9" width="25.375" style="2" customWidth="1"/>
     <col min="10" max="16384" width="9" style="2"/>
   </cols>
@@ -1467,7 +1482,7 @@
       </c>
     </row>
     <row r="2" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1495,167 +1510,158 @@
         <v>271</v>
       </c>
       <c r="J2" s="3"/>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
     </row>
     <row r="3" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="15"/>
-      <c r="D3" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>262</v>
+      <c r="A3" s="16"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="5" t="s">
+        <v>287</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
     </row>
     <row r="4" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="15"/>
+      <c r="A4" s="16"/>
       <c r="D4" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="3"/>
-      <c r="K4" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
     </row>
     <row r="5" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="15"/>
-      <c r="B5" s="1" t="s">
-        <v>250</v>
-      </c>
+      <c r="A5" s="16"/>
       <c r="D5" s="1" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>245</v>
+        <v>267</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>263</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="3"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
+      <c r="K5" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
     </row>
     <row r="6" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="15"/>
-      <c r="E6" s="10" t="s">
+      <c r="A6" s="16"/>
+      <c r="B6" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+    </row>
+    <row r="7" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="16"/>
+      <c r="E7" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F7" s="12" t="s">
         <v>258</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H7" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="I6" s="10"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-    </row>
-    <row r="7" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="15"/>
-      <c r="B7" s="11" t="s">
+      <c r="I7" s="10"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+    </row>
+    <row r="8" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="16"/>
+      <c r="B8" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C8" s="11" t="s">
         <v>235</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D8" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E8" s="11" t="s">
         <v>236</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F8" s="11" t="s">
         <v>242</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G8" s="11" t="s">
         <v>240</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H8" s="11" t="s">
         <v>241</v>
-      </c>
-      <c r="I7" s="11"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-    </row>
-    <row r="8" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="15"/>
-      <c r="B8" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>244</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>237</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>243</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>238</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>239</v>
       </c>
       <c r="I8" s="11"/>
       <c r="K8" s="4"/>
@@ -1665,297 +1671,311 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="15"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="I9" s="11"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
     </row>
     <row r="10" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="15"/>
+      <c r="A10" s="16"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
-      <c r="D10" s="1" t="s">
-        <v>274</v>
+      <c r="D10" s="2" t="s">
+        <v>273</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="F10" s="1"/>
+        <v>191</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>284</v>
+      </c>
       <c r="G10" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K10" s="13"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
+        <v>6</v>
+      </c>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="14"/>
     </row>
     <row r="11" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="15"/>
+      <c r="A11" s="16"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
+        <v>7</v>
+      </c>
+      <c r="K11" s="14"/>
+      <c r="L11" s="14"/>
+      <c r="M11" s="14"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="14"/>
     </row>
     <row r="12" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="15"/>
+      <c r="A12" s="16"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K12" s="13"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="13"/>
+        <v>8</v>
+      </c>
+      <c r="K12" s="14"/>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
+      <c r="N12" s="14"/>
+      <c r="O12" s="14"/>
     </row>
     <row r="13" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="15"/>
+      <c r="A13" s="16"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
+        <v>9</v>
+      </c>
+      <c r="K13" s="14"/>
+      <c r="L13" s="14"/>
+      <c r="M13" s="14"/>
+      <c r="N13" s="14"/>
+      <c r="O13" s="14"/>
     </row>
     <row r="14" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="15"/>
+      <c r="A14" s="16"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K14" s="13"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
+        <v>10</v>
+      </c>
+      <c r="K14" s="14"/>
+      <c r="L14" s="14"/>
+      <c r="M14" s="14"/>
+      <c r="N14" s="14"/>
+      <c r="O14" s="14"/>
     </row>
     <row r="15" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="15"/>
+      <c r="A15" s="16"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>11</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
+      <c r="M15" s="14"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="14"/>
     </row>
     <row r="16" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="15"/>
+      <c r="A16" s="16"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>272</v>
+        <v>197</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>72</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="15"/>
+      <c r="A17" s="16"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>198</v>
+        <v>272</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="15"/>
+      <c r="A18" s="16"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="15"/>
+      <c r="A19" s="16"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>12</v>
+        <v>74</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>12</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="15"/>
+      <c r="A20" s="16"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
+      <c r="D20" s="1" t="s">
+        <v>283</v>
+      </c>
       <c r="E20" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="15"/>
+      <c r="A21" s="16"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="15"/>
+      <c r="A22" s="16"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
-        <v>126</v>
+        <v>202</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="15"/>
+      <c r="A23" s="16"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>203</v>
+        <v>126</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>75</v>
+        <v>15</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>75</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1964,30 +1984,30 @@
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="17"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="H25" s="1" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1996,30 +2016,30 @@
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
       <c r="E27" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -2028,14 +2048,14 @@
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
@@ -2044,14 +2064,14 @@
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
       <c r="E29" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="6" t="s">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>76</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -2060,14 +2080,14 @@
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
       <c r="E30" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="6" t="s">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>21</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -2076,14 +2096,14 @@
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
       <c r="E31" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
@@ -2092,14 +2112,14 @@
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
       <c r="E32" s="6" t="s">
-        <v>127</v>
+        <v>211</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
@@ -2108,14 +2128,14 @@
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
       <c r="E33" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -2124,14 +2144,14 @@
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6" t="s">
-        <v>212</v>
+        <v>128</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
@@ -2140,14 +2160,14 @@
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
       <c r="E35" s="6" t="s">
-        <v>129</v>
+        <v>212</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="6" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
@@ -2156,14 +2176,14 @@
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
       <c r="E36" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
@@ -2172,14 +2192,14 @@
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
       <c r="E37" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
@@ -2188,14 +2208,14 @@
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
       <c r="E38" s="6" t="s">
-        <v>213</v>
+        <v>131</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="6" t="s">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>26</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
@@ -2204,14 +2224,14 @@
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
       <c r="E39" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -2220,14 +2240,14 @@
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
       <c r="E40" s="6" t="s">
-        <v>132</v>
+        <v>214</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="6" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
@@ -2236,14 +2256,14 @@
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
       <c r="E41" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6" t="s">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>28</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
@@ -2252,14 +2272,14 @@
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
       <c r="E42" s="6" t="s">
-        <v>215</v>
+        <v>133</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="6" t="s">
-        <v>81</v>
+        <v>28</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>81</v>
+        <v>28</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -2268,14 +2288,14 @@
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
       <c r="E43" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -2284,14 +2304,14 @@
       <c r="C44" s="6"/>
       <c r="D44" s="6"/>
       <c r="E44" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="6" t="s">
-        <v>29</v>
+        <v>82</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
@@ -2300,14 +2320,14 @@
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
       <c r="E45" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="6" t="s">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>84</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -2316,14 +2336,14 @@
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
       <c r="E46" s="6" t="s">
-        <v>134</v>
+        <v>218</v>
       </c>
       <c r="F46" s="6"/>
       <c r="G46" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -2332,14 +2352,14 @@
       <c r="C47" s="6"/>
       <c r="D47" s="6"/>
       <c r="E47" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="6" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
@@ -2348,14 +2368,14 @@
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
       <c r="E48" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
@@ -2364,14 +2384,14 @@
       <c r="C49" s="6"/>
       <c r="D49" s="6"/>
       <c r="E49" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F49" s="6"/>
       <c r="G49" s="6" t="s">
-        <v>86</v>
+        <v>31</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>86</v>
+        <v>31</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
@@ -2380,14 +2400,14 @@
       <c r="C50" s="6"/>
       <c r="D50" s="6"/>
       <c r="E50" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="6" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
@@ -2396,14 +2416,14 @@
       <c r="C51" s="6"/>
       <c r="D51" s="6"/>
       <c r="E51" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F51" s="6"/>
       <c r="G51" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
@@ -2412,14 +2432,14 @@
       <c r="C52" s="6"/>
       <c r="D52" s="6"/>
       <c r="E52" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
@@ -2428,14 +2448,14 @@
       <c r="C53" s="6"/>
       <c r="D53" s="6"/>
       <c r="E53" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F53" s="6"/>
       <c r="G53" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
@@ -2444,14 +2464,14 @@
       <c r="C54" s="6"/>
       <c r="D54" s="6"/>
       <c r="E54" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F54" s="6"/>
       <c r="G54" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
@@ -2460,14 +2480,14 @@
       <c r="C55" s="6"/>
       <c r="D55" s="6"/>
       <c r="E55" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F55" s="6"/>
       <c r="G55" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
@@ -2476,14 +2496,14 @@
       <c r="C56" s="6"/>
       <c r="D56" s="6"/>
       <c r="E56" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F56" s="6"/>
       <c r="G56" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
@@ -2492,14 +2512,14 @@
       <c r="C57" s="6"/>
       <c r="D57" s="6"/>
       <c r="E57" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F57" s="6"/>
       <c r="G57" s="6" t="s">
-        <v>87</v>
+        <v>38</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>87</v>
+        <v>38</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
@@ -2508,14 +2528,14 @@
       <c r="C58" s="6"/>
       <c r="D58" s="6"/>
       <c r="E58" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F58" s="6"/>
       <c r="G58" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
@@ -2524,14 +2544,14 @@
       <c r="C59" s="6"/>
       <c r="D59" s="6"/>
       <c r="E59" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F59" s="6"/>
       <c r="G59" s="6" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
@@ -2540,14 +2560,14 @@
       <c r="C60" s="6"/>
       <c r="D60" s="6"/>
       <c r="E60" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F60" s="6"/>
       <c r="G60" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -2556,14 +2576,14 @@
       <c r="C61" s="6"/>
       <c r="D61" s="6"/>
       <c r="E61" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F61" s="6"/>
       <c r="G61" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
@@ -2572,14 +2592,14 @@
       <c r="C62" s="6"/>
       <c r="D62" s="6"/>
       <c r="E62" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F62" s="6"/>
       <c r="G62" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
@@ -2588,14 +2608,14 @@
       <c r="C63" s="6"/>
       <c r="D63" s="6"/>
       <c r="E63" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F63" s="6"/>
       <c r="G63" s="6" t="s">
-        <v>286</v>
+        <v>42</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
@@ -2604,14 +2624,14 @@
       <c r="C64" s="6"/>
       <c r="D64" s="6"/>
       <c r="E64" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F64" s="6"/>
       <c r="G64" s="6" t="s">
-        <v>44</v>
+        <v>286</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
@@ -2620,14 +2640,14 @@
       <c r="C65" s="6"/>
       <c r="D65" s="6"/>
       <c r="E65" s="6" t="s">
-        <v>219</v>
+        <v>152</v>
       </c>
       <c r="F65" s="6"/>
       <c r="G65" s="6" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>90</v>
+        <v>44</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
@@ -2636,14 +2656,14 @@
       <c r="C66" s="6"/>
       <c r="D66" s="6"/>
       <c r="E66" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F66" s="6"/>
       <c r="G66" s="6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
@@ -2652,14 +2672,14 @@
       <c r="C67" s="6"/>
       <c r="D67" s="6"/>
       <c r="E67" s="6" t="s">
-        <v>153</v>
+        <v>220</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
@@ -2668,14 +2688,14 @@
       <c r="C68" s="6"/>
       <c r="D68" s="6"/>
       <c r="E68" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F68" s="6"/>
       <c r="G68" s="6" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
@@ -2684,14 +2704,14 @@
       <c r="C69" s="6"/>
       <c r="D69" s="6"/>
       <c r="E69" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F69" s="6"/>
       <c r="G69" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -2700,14 +2720,14 @@
       <c r="C70" s="6"/>
       <c r="D70" s="6"/>
       <c r="E70" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F70" s="6"/>
       <c r="G70" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
@@ -2716,14 +2736,14 @@
       <c r="C71" s="6"/>
       <c r="D71" s="6"/>
       <c r="E71" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F71" s="6"/>
       <c r="G71" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
@@ -2732,14 +2752,14 @@
       <c r="C72" s="6"/>
       <c r="D72" s="6"/>
       <c r="E72" s="6" t="s">
-        <v>221</v>
+        <v>157</v>
       </c>
       <c r="F72" s="6"/>
       <c r="G72" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
@@ -2748,14 +2768,14 @@
       <c r="C73" s="6"/>
       <c r="D73" s="6"/>
       <c r="E73" s="6" t="s">
-        <v>158</v>
+        <v>221</v>
       </c>
       <c r="F73" s="6"/>
       <c r="G73" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
@@ -2764,14 +2784,14 @@
       <c r="C74" s="6"/>
       <c r="D74" s="6"/>
       <c r="E74" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F74" s="6"/>
       <c r="G74" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
@@ -2780,14 +2800,14 @@
       <c r="C75" s="6"/>
       <c r="D75" s="6"/>
       <c r="E75" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F75" s="6"/>
       <c r="G75" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
@@ -2796,14 +2816,14 @@
       <c r="C76" s="6"/>
       <c r="D76" s="6"/>
       <c r="E76" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F76" s="6"/>
       <c r="G76" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
@@ -2812,14 +2832,14 @@
       <c r="C77" s="6"/>
       <c r="D77" s="6"/>
       <c r="E77" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F77" s="6"/>
       <c r="G77" s="6" t="s">
-        <v>94</v>
+        <v>53</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>94</v>
+        <v>53</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
@@ -2828,14 +2848,14 @@
       <c r="C78" s="6"/>
       <c r="D78" s="6"/>
       <c r="E78" s="6" t="s">
-        <v>222</v>
+        <v>162</v>
       </c>
       <c r="F78" s="6"/>
       <c r="G78" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
@@ -2844,14 +2864,14 @@
       <c r="C79" s="6"/>
       <c r="D79" s="6"/>
       <c r="E79" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F79" s="6"/>
       <c r="G79" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
@@ -2860,14 +2880,14 @@
       <c r="C80" s="6"/>
       <c r="D80" s="6"/>
       <c r="E80" s="6" t="s">
-        <v>163</v>
+        <v>223</v>
       </c>
       <c r="F80" s="6"/>
       <c r="G80" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.2">
@@ -2876,14 +2896,14 @@
       <c r="C81" s="6"/>
       <c r="D81" s="6"/>
       <c r="E81" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F81" s="6"/>
       <c r="G81" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H81" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.2">
@@ -2892,14 +2912,14 @@
       <c r="C82" s="6"/>
       <c r="D82" s="6"/>
       <c r="E82" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F82" s="6"/>
       <c r="G82" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>54</v>
+        <v>102</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.2">
@@ -2908,14 +2928,14 @@
       <c r="C83" s="6"/>
       <c r="D83" s="6"/>
       <c r="E83" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F83" s="6"/>
       <c r="G83" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H83" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.2">
@@ -2924,14 +2944,14 @@
       <c r="C84" s="6"/>
       <c r="D84" s="6"/>
       <c r="E84" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F84" s="6"/>
       <c r="G84" s="6" t="s">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>103</v>
+        <v>55</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
@@ -2940,14 +2960,14 @@
       <c r="C85" s="6"/>
       <c r="D85" s="6"/>
       <c r="E85" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F85" s="6"/>
       <c r="G85" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.2">
@@ -2956,14 +2976,14 @@
       <c r="C86" s="6"/>
       <c r="D86" s="6"/>
       <c r="E86" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F86" s="6"/>
       <c r="G86" s="6" t="s">
-        <v>103</v>
+        <v>55</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
@@ -2972,14 +2992,14 @@
       <c r="C87" s="6"/>
       <c r="D87" s="6"/>
       <c r="E87" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F87" s="6"/>
       <c r="G87" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>56</v>
+        <v>105</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.2">
@@ -2988,14 +3008,14 @@
       <c r="C88" s="6"/>
       <c r="D88" s="6"/>
       <c r="E88" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F88" s="6"/>
       <c r="G88" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.2">
@@ -3004,14 +3024,14 @@
       <c r="C89" s="6"/>
       <c r="D89" s="6"/>
       <c r="E89" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F89" s="6"/>
       <c r="G89" s="6" t="s">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="H89" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.2">
@@ -3020,14 +3040,14 @@
       <c r="C90" s="6"/>
       <c r="D90" s="6"/>
       <c r="E90" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F90" s="6"/>
       <c r="G90" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.2">
@@ -3036,14 +3056,14 @@
       <c r="C91" s="6"/>
       <c r="D91" s="6"/>
       <c r="E91" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F91" s="6"/>
       <c r="G91" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.2">
@@ -3052,14 +3072,14 @@
       <c r="C92" s="6"/>
       <c r="D92" s="6"/>
       <c r="E92" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F92" s="6"/>
       <c r="G92" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.2">
@@ -3068,14 +3088,14 @@
       <c r="C93" s="6"/>
       <c r="D93" s="6"/>
       <c r="E93" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F93" s="6"/>
       <c r="G93" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.2">
@@ -3084,14 +3104,14 @@
       <c r="C94" s="6"/>
       <c r="D94" s="6"/>
       <c r="E94" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F94" s="6"/>
       <c r="G94" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>106</v>
+        <v>62</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.2">
@@ -3100,14 +3120,14 @@
       <c r="C95" s="6"/>
       <c r="D95" s="6"/>
       <c r="E95" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F95" s="6"/>
       <c r="G95" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H95" s="6" t="s">
-        <v>63</v>
+        <v>106</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.2">
@@ -3116,14 +3136,14 @@
       <c r="C96" s="6"/>
       <c r="D96" s="6"/>
       <c r="E96" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F96" s="6"/>
       <c r="G96" s="6" t="s">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.2">
@@ -3132,14 +3152,14 @@
       <c r="C97" s="6"/>
       <c r="D97" s="6"/>
       <c r="E97" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F97" s="6"/>
       <c r="G97" s="6" t="s">
-        <v>63</v>
+        <v>106</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.2">
@@ -3148,14 +3168,14 @@
       <c r="C98" s="6"/>
       <c r="D98" s="6"/>
       <c r="E98" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F98" s="6"/>
       <c r="G98" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.2">
@@ -3164,14 +3184,14 @@
       <c r="C99" s="6"/>
       <c r="D99" s="6"/>
       <c r="E99" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F99" s="6"/>
       <c r="G99" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H99" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.2">
@@ -3180,14 +3200,14 @@
       <c r="C100" s="6"/>
       <c r="D100" s="6"/>
       <c r="E100" s="6" t="s">
-        <v>224</v>
+        <v>182</v>
       </c>
       <c r="F100" s="6"/>
       <c r="G100" s="6" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.2">
@@ -3196,14 +3216,14 @@
       <c r="C101" s="6"/>
       <c r="D101" s="6"/>
       <c r="E101" s="6" t="s">
-        <v>183</v>
+        <v>224</v>
       </c>
       <c r="F101" s="6"/>
       <c r="G101" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H101" s="6" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.2">
@@ -3212,14 +3232,14 @@
       <c r="C102" s="6"/>
       <c r="D102" s="6"/>
       <c r="E102" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F102" s="6"/>
       <c r="G102" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>112</v>
+        <v>66</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.2">
@@ -3228,14 +3248,14 @@
       <c r="C103" s="6"/>
       <c r="D103" s="6"/>
       <c r="E103" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F103" s="6"/>
       <c r="G103" s="6" t="s">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="H103" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.2">
@@ -3244,14 +3264,14 @@
       <c r="C104" s="6"/>
       <c r="D104" s="6"/>
       <c r="E104" s="6" t="s">
-        <v>225</v>
+        <v>185</v>
       </c>
       <c r="F104" s="6"/>
       <c r="G104" s="6" t="s">
-        <v>112</v>
+        <v>66</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.2">
@@ -3260,14 +3280,14 @@
       <c r="C105" s="6"/>
       <c r="D105" s="6"/>
       <c r="E105" s="6" t="s">
-        <v>186</v>
+        <v>225</v>
       </c>
       <c r="F105" s="6"/>
       <c r="G105" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H105" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.2">
@@ -3276,14 +3296,14 @@
       <c r="C106" s="6"/>
       <c r="D106" s="6"/>
       <c r="E106" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F106" s="6"/>
       <c r="G106" s="6" t="s">
-        <v>67</v>
+        <v>113</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.2">
@@ -3292,14 +3312,14 @@
       <c r="C107" s="6"/>
       <c r="D107" s="6"/>
       <c r="E107" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F107" s="6"/>
       <c r="G107" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H107" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.2">
@@ -3308,14 +3328,14 @@
       <c r="C108" s="6"/>
       <c r="D108" s="6"/>
       <c r="E108" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F108" s="6"/>
       <c r="G108" s="6" t="s">
-        <v>116</v>
+        <v>68</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.2">
@@ -3324,14 +3344,14 @@
       <c r="C109" s="6"/>
       <c r="D109" s="6"/>
       <c r="E109" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F109" s="6"/>
       <c r="G109" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H109" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.2">
@@ -3340,14 +3360,14 @@
       <c r="C110" s="6"/>
       <c r="D110" s="6"/>
       <c r="E110" s="6" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="F110" s="6"/>
       <c r="G110" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H110" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.2">
@@ -3356,14 +3376,14 @@
       <c r="C111" s="6"/>
       <c r="D111" s="6"/>
       <c r="E111" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F111" s="6"/>
       <c r="G111" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H111" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.2">
@@ -3372,14 +3392,14 @@
       <c r="C112" s="6"/>
       <c r="D112" s="6"/>
       <c r="E112" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F112" s="6"/>
       <c r="G112" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H112" s="6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.2">
@@ -3388,14 +3408,14 @@
       <c r="C113" s="6"/>
       <c r="D113" s="6"/>
       <c r="E113" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F113" s="6"/>
       <c r="G113" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H113" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.2">
@@ -3404,14 +3424,14 @@
       <c r="C114" s="6"/>
       <c r="D114" s="6"/>
       <c r="E114" s="6" t="s">
-        <v>125</v>
+        <v>229</v>
       </c>
       <c r="F114" s="6"/>
       <c r="G114" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H114" s="6" t="s">
-        <v>285</v>
+        <v>125</v>
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.2">
@@ -3419,12 +3439,16 @@
       <c r="B115" s="6"/>
       <c r="C115" s="6"/>
       <c r="D115" s="6"/>
-      <c r="E115" s="6"/>
+      <c r="E115" s="6" t="s">
+        <v>125</v>
+      </c>
       <c r="F115" s="6"/>
       <c r="G115" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="H115" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="H115" s="6" t="s">
+        <v>285</v>
+      </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A116" s="6"/>
@@ -3434,23 +3458,35 @@
       <c r="E116" s="6"/>
       <c r="F116" s="6"/>
       <c r="G116" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H116" s="6"/>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A117" s="6"/>
+      <c r="B117" s="6"/>
+      <c r="C117" s="6"/>
+      <c r="D117" s="6"/>
+      <c r="E117" s="6"/>
+      <c r="F117" s="6"/>
+      <c r="G117" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="H116" s="6"/>
+      <c r="H117" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="K11:O11"/>
     <mergeCell ref="K12:O12"/>
     <mergeCell ref="K13:O13"/>
     <mergeCell ref="K14:O14"/>
-    <mergeCell ref="A2:A24"/>
+    <mergeCell ref="K15:O15"/>
+    <mergeCell ref="A2:A25"/>
     <mergeCell ref="K2:O2"/>
-    <mergeCell ref="K4:O4"/>
     <mergeCell ref="K5:O5"/>
     <mergeCell ref="K6:O6"/>
-    <mergeCell ref="K9:O9"/>
+    <mergeCell ref="K7:O7"/>
     <mergeCell ref="K10:O10"/>
+    <mergeCell ref="K11:O11"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>